<commit_message>
Daily NSE scan: 2026-09-09
</commit_message>
<xml_diff>
--- a/output/2026-09-09/enriched_analysis.xlsx
+++ b/output/2026-09-09/enriched_analysis.xlsx
@@ -793,27 +793,27 @@
         <v>265.85</v>
       </c>
       <c r="J2" t="n">
-        <v>158.6</v>
+        <v>189.03</v>
       </c>
       <c r="K2" t="n">
-        <v>67.59999999999999</v>
+        <v>40.6</v>
       </c>
       <c r="L2" t="n">
         <v>64.63</v>
       </c>
       <c r="M2" t="n">
-        <v>1.99</v>
+        <v>3.32</v>
       </c>
       <c r="N2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>16-06-2026</t>
+          <t>08-09-2026</t>
         </is>
       </c>
       <c r="P2" t="n">
-        <v>0.077</v>
+        <v>0.128</v>
       </c>
       <c r="Q2" t="n">
         <v>2601</v>
@@ -855,19 +855,19 @@
         <v>97.7</v>
       </c>
       <c r="AD2" t="n">
-        <v>158.5989279295042</v>
+        <v>189.0309324107478</v>
       </c>
       <c r="AE2" t="n">
-        <v>67.59999999999999</v>
+        <v>40.6</v>
       </c>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>Stale</t>
+          <t>Fresh</t>
         </is>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
-          <t>Stale Accumulation</t>
+          <t>Confirmed Accumulation</t>
         </is>
       </c>
       <c r="AH2" t="inlineStr">
@@ -882,53 +882,53 @@
       </c>
       <c r="AJ2" t="inlineStr">
         <is>
-          <t>16-06-2026</t>
+          <t>08-09-2026</t>
         </is>
       </c>
       <c r="AK2" t="n">
-        <v>8</v>
+        <v>92</v>
       </c>
       <c r="AL2" t="n">
         <v>93</v>
       </c>
       <c r="AM2" t="n">
-        <v>85</v>
+        <v>1</v>
       </c>
       <c r="AN2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AO2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AP2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AQ2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AR2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AS2" t="n">
-        <v>0</v>
+        <v>13278006</v>
       </c>
       <c r="AT2" t="n">
-        <v>0</v>
+        <v>13278006</v>
       </c>
       <c r="AU2" t="n">
-        <v>0</v>
+        <v>13278006</v>
       </c>
       <c r="AV2" t="n">
-        <v>0</v>
+        <v>13278006</v>
       </c>
       <c r="AW2" t="n">
-        <v>7976605</v>
+        <v>21254611</v>
       </c>
       <c r="AX2" t="n">
-        <v>0</v>
+        <v>13278006</v>
       </c>
       <c r="AY2" t="n">
-        <v>0</v>
+        <v>13278006</v>
       </c>
       <c r="AZ2" t="n">
         <v>1</v>
@@ -937,7 +937,7 @@
         <v>0</v>
       </c>
       <c r="BB2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -9735,23 +9735,23 @@
         <v>265.85</v>
       </c>
       <c r="D2" t="n">
-        <v>158.6</v>
+        <v>189.03</v>
       </c>
       <c r="E2" t="n">
-        <v>67.59999999999999</v>
+        <v>40.6</v>
       </c>
       <c r="F2" t="n">
         <v>64.63</v>
       </c>
       <c r="G2" t="n">
-        <v>1.99</v>
+        <v>3.32</v>
       </c>
       <c r="H2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>16-06-2026</t>
+          <t>08-09-2026</t>
         </is>
       </c>
     </row>

</xml_diff>